<commit_message>
Add word "Overvej" to Sange.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Sange.xlsx
+++ b/12-06-2026-vokab/Sange.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V1"/>
+  <dimension ref="A1:V2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -493,9 +493,77 @@
         <v>Lapses</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>08d1490d-acfa-4570-a2a4-a2e4ed38227c</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Overvej</v>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+      <c r="E2" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v>-r, -de, -tBøjningsformerovervejerovervejedeovervejet</v>
+      </c>
+      <c r="H2" t="str">
+        <v>[-ˌvɑjˀə]</v>
+      </c>
+      <c r="I2" t="str">
+        <v>https://static.ordnet.dk/mp3/11038/11038552_1.mp3</v>
+      </c>
+      <c r="J2" t="str">
+        <v>tænke over noget eller tænke på at gøre noget idet man vurderer hvad der taler for og imodSynonymer tænke igennemgennemtænkeOrd i nærhedenovervejetænke over tingeneanalysere situationenvurdere situationentage temperaturen på nogetgå i tænkeboksgenove</v>
+      </c>
+      <c r="K2" t="str">
+        <v>Consider</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Overvej om ikke du vil sige noget til en af sangene.</v>
+      </c>
+      <c r="M2" t="str">
+        <v>(5) Fællesklang Sønderborg | Facebook</v>
+      </c>
+      <c r="N2" t="str">
+        <v>https://www.facebook.com/groups/9417595711665677</v>
+      </c>
+      <c r="O2" t="str">
+        <v>https://www.facebook.com/groups/9417595711665677#:~:text=Overvej</v>
+      </c>
+      <c r="P2" t="str">
+        <v/>
+      </c>
+      <c r="Q2" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R2" t="str">
+        <v/>
+      </c>
+      <c r="S2" t="str">
+        <v/>
+      </c>
+      <c r="T2" t="str">
+        <v/>
+      </c>
+      <c r="U2" t="str">
+        <v/>
+      </c>
+      <c r="V2" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -504,22 +572,22 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:P1"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="36.83203125" customWidth="1"/>
-    <col min="5" max="5" width="36.83203125" customWidth="1"/>
-    <col min="6" max="6" width="50.83203125" customWidth="1"/>
-    <col min="7" max="7" width="24.83203125" customWidth="1"/>
-    <col min="8" max="8" width="24.83203125" customWidth="1"/>
-    <col min="9" max="9" width="24.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" customWidth="1"/>
-    <col min="12" max="12" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="13" max="13" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="14" max="14" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="15" max="15" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="16" max="16" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="30.83203125"/>
+    <col min="4" max="4" customWidth="1" width="36.83203125"/>
+    <col min="5" max="5" customWidth="1" width="36.83203125"/>
+    <col min="6" max="6" customWidth="1" width="50.83203125"/>
+    <col min="7" max="7" customWidth="1" width="24.83203125"/>
+    <col min="8" max="8" customWidth="1" width="24.83203125"/>
+    <col min="9" max="9" customWidth="1" width="24.83203125"/>
+    <col min="10" max="10" customWidth="1" width="18.83203125"/>
+    <col min="11" max="11" customWidth="1" width="10.83203125"/>
+    <col min="12" max="12" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="13" max="13" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="14" max="14" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="15" max="15" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="16" max="16" customWidth="1" width="7.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -583,8 +651,8 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B4"/>
   <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+    <col min="1" max="1" customWidth="1" width="16.83203125"/>
+    <col min="2" max="2" customWidth="1" width="28.83203125"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Add word "elnettet" to Sange.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Sange.xlsx
+++ b/12-06-2026-vokab/Sange.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
-        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
-        <a:font script="Hans" typeface="å®ä½"/>
-        <a:font script="Hant" typeface="æ°ç´°æé«"/>
+        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
+        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
+        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
+        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
-        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
-        <a:font script="Hans" typeface="å®ä½"/>
-        <a:font script="Hant" typeface="æ°ç´°æé«"/>
+        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
+        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
+        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
+        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V2"/>
+  <dimension ref="A1:V3"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -561,9 +561,77 @@
         <v/>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>e427b635-8083-4bd3-be4c-e41438960d8d</v>
+      </c>
+      <c r="B3" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="C3" t="str">
+        <v>elnettet</v>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
+      <c r="K3" t="str">
+        <v>the mains</v>
+      </c>
+      <c r="L3" t="str">
+        <v>Første af sin slags i Europa: Printplade i danskeres varmepumper aflaster elnettet</v>
+      </c>
+      <c r="M3" t="str">
+        <v>Ingeniøren - nyheder om teknologi og samfund</v>
+      </c>
+      <c r="N3" t="str">
+        <v>https://ing.dk/</v>
+      </c>
+      <c r="O3" t="str">
+        <v>https://ing.dk/#:~:text=elnettet</v>
+      </c>
+      <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
+        <v>pending</v>
+      </c>
+      <c r="R3" t="str">
+        <v/>
+      </c>
+      <c r="S3" t="str">
+        <v/>
+      </c>
+      <c r="T3" t="str">
+        <v/>
+      </c>
+      <c r="U3" t="str">
+        <v/>
+      </c>
+      <c r="V3" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V3"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Phone: add 1 entry in Sange.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Sange.xlsx
+++ b/12-06-2026-vokab/Sange.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
-        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
-        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
-        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
+        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
-        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
-        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
-        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
+        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V3"/>
+  <dimension ref="A1:W4"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -423,6 +423,7 @@
     <col min="20" max="20" width="7.83203125" customWidth="1" hidden="true"/>
     <col min="21" max="21" width="6.83203125" customWidth="1" hidden="true"/>
     <col min="22" max="22" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="23" max="23" width="40.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -492,6 +493,9 @@
       <c r="V1" t="str">
         <v>Lapses</v>
       </c>
+      <c r="W1" t="str">
+        <v>Candidates</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -629,33 +633,105 @@
         <v/>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>c57cd97f-b6d3-4c65-97d9-9cc4fdfdf720</v>
+      </c>
+      <c r="B4" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="C4" t="str">
+        <v>rodet</v>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v/>
+      </c>
+      <c r="N4" t="str">
+        <v/>
+      </c>
+      <c r="O4" t="str">
+        <v/>
+      </c>
+      <c r="P4" t="str">
+        <v/>
+      </c>
+      <c r="Q4" t="str">
+        <v>pending</v>
+      </c>
+      <c r="R4" t="str">
+        <v/>
+      </c>
+      <c r="S4" t="str">
+        <v/>
+      </c>
+      <c r="T4" t="str">
+        <v/>
+      </c>
+      <c r="U4" t="str">
+        <v/>
+      </c>
+      <c r="V4" t="str">
+        <v/>
+      </c>
+      <c r="W4" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:Q1"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="30.83203125"/>
-    <col min="4" max="4" customWidth="1" width="36.83203125"/>
-    <col min="5" max="5" customWidth="1" width="36.83203125"/>
-    <col min="6" max="6" customWidth="1" width="50.83203125"/>
-    <col min="7" max="7" customWidth="1" width="24.83203125"/>
-    <col min="8" max="8" customWidth="1" width="24.83203125"/>
-    <col min="9" max="9" customWidth="1" width="24.83203125"/>
-    <col min="10" max="10" customWidth="1" width="18.83203125"/>
-    <col min="11" max="11" customWidth="1" width="10.83203125"/>
-    <col min="12" max="12" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="13" max="13" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="14" max="14" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="15" max="15" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="16" max="16" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col min="4" max="4" width="36.83203125" customWidth="1"/>
+    <col min="5" max="5" width="36.83203125" customWidth="1"/>
+    <col min="6" max="6" width="50.83203125" customWidth="1"/>
+    <col min="7" max="7" width="24.83203125" customWidth="1"/>
+    <col min="8" max="8" width="24.83203125" customWidth="1"/>
+    <col min="9" max="9" width="24.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="10.83203125" customWidth="1"/>
+    <col min="12" max="12" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="13" max="13" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="14" max="14" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="15" max="15" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="16" max="16" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="17" max="17" width="40.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -707,10 +783,13 @@
       <c r="P1" t="str">
         <v>Lapses</v>
       </c>
+      <c r="Q1" t="str">
+        <v>Candidates</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Phone: progress for 1 card in Sange.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Sange.xlsx
+++ b/12-06-2026-vokab/Sange.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -401,29 +401,29 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:W6"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="36.83203125" customWidth="1"/>
-    <col min="11" max="11" width="36.83203125" customWidth="1"/>
-    <col min="12" max="12" width="50.83203125" customWidth="1"/>
-    <col min="13" max="13" width="24.83203125" customWidth="1"/>
-    <col min="14" max="14" width="24.83203125" customWidth="1"/>
-    <col min="15" max="15" width="24.83203125" customWidth="1"/>
-    <col min="16" max="16" width="18.83203125" customWidth="1"/>
-    <col min="17" max="17" width="10.83203125" customWidth="1"/>
-    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="23" max="23" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="18.83203125"/>
+    <col min="4" max="4" customWidth="1" width="14.83203125"/>
+    <col min="5" max="5" customWidth="1" width="11.83203125"/>
+    <col min="6" max="6" customWidth="1" width="8.83203125"/>
+    <col min="7" max="7" customWidth="1" width="26.83203125"/>
+    <col min="8" max="8" customWidth="1" width="16.83203125"/>
+    <col min="9" max="9" customWidth="1" width="18.83203125"/>
+    <col min="10" max="10" customWidth="1" width="36.83203125"/>
+    <col min="11" max="11" customWidth="1" width="36.83203125"/>
+    <col min="12" max="12" customWidth="1" width="50.83203125"/>
+    <col min="13" max="13" customWidth="1" width="24.83203125"/>
+    <col min="14" max="14" customWidth="1" width="24.83203125"/>
+    <col min="15" max="15" customWidth="1" width="24.83203125"/>
+    <col min="16" max="16" customWidth="1" width="18.83203125"/>
+    <col min="17" max="17" customWidth="1" width="10.83203125"/>
+    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="23" max="23" customWidth="1" width="40.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -686,19 +686,19 @@
         <v>pending</v>
       </c>
       <c r="R4" t="str">
-        <v/>
+        <v>2026-06-15</v>
       </c>
       <c r="S4" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="T4" t="str">
-        <v/>
+        <v>2.3</v>
       </c>
       <c r="U4" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="V4" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="W4" t="str">
         <v/>

</xml_diff>

<commit_message>
Enrich 4 pending entries in Sange.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Sange.xlsx
+++ b/12-06-2026-vokab/Sange.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -576,25 +576,25 @@
         <v>elnettet</v>
       </c>
       <c r="D3" t="str">
-        <v/>
+        <v>elnet</v>
       </c>
       <c r="E3" t="str">
-        <v/>
+        <v>substantiv</v>
       </c>
       <c r="F3" t="str">
-        <v/>
+        <v>et</v>
       </c>
       <c r="G3" t="str">
-        <v/>
+        <v>-tet, -, -tene</v>
       </c>
       <c r="H3" t="str">
-        <v/>
+        <v>[ˈεl-]</v>
       </c>
       <c r="I3" t="str">
-        <v/>
+        <v>https://static.ordnet.dk/mp3/41000/41000648_1.mp3</v>
       </c>
       <c r="J3" t="str">
-        <v/>
+        <v>system af kabler, ledninger, transformatorstationer m.m. der forbinder ét eller flere kraftværker eller andre elektricitetsproducerende anlæg med forbrugerne af elektriciteten</v>
       </c>
       <c r="K3" t="str">
         <v>the mains</v>
@@ -615,7 +615,7 @@
         <v/>
       </c>
       <c r="Q3" t="str">
-        <v>pending</v>
+        <v>ok</v>
       </c>
       <c r="R3" t="str">
         <v/>
@@ -630,6 +630,9 @@
         <v/>
       </c>
       <c r="V3" t="str">
+        <v/>
+      </c>
+      <c r="W3" t="str">
         <v/>
       </c>
     </row>
@@ -644,28 +647,28 @@
         <v>rodet</v>
       </c>
       <c r="D4" t="str">
-        <v/>
+        <v>rodet</v>
       </c>
       <c r="E4" t="str">
-        <v/>
+        <v>adjektiv</v>
       </c>
       <c r="F4" t="str">
         <v/>
       </c>
       <c r="G4" t="str">
-        <v/>
+        <v>-, rodede</v>
       </c>
       <c r="H4" t="str">
-        <v/>
+        <v>[ˈʁoːðəd]</v>
       </c>
       <c r="I4" t="str">
-        <v/>
+        <v>https://static.ordnet.dk/mp3/11043/11043541_1.mp3</v>
       </c>
       <c r="J4" t="str">
-        <v/>
+        <v>med mange ting som ikke er lagt på plads, eller som er anbragt uordentligt</v>
       </c>
       <c r="K4" t="str">
-        <v/>
+        <v>messy</v>
       </c>
       <c r="L4" t="str">
         <v/>
@@ -683,7 +686,7 @@
         <v/>
       </c>
       <c r="Q4" t="str">
-        <v>pending</v>
+        <v>ok</v>
       </c>
       <c r="R4" t="str">
         <v>2026-06-15</v>
@@ -715,28 +718,28 @@
         <v>opløse</v>
       </c>
       <c r="D5" t="str">
-        <v/>
+        <v>opløse</v>
       </c>
       <c r="E5" t="str">
-        <v/>
+        <v>verbum</v>
       </c>
       <c r="F5" t="str">
         <v/>
       </c>
       <c r="G5" t="str">
-        <v/>
+        <v>-r, opløste, opløst</v>
       </c>
       <c r="H5" t="str">
-        <v/>
+        <v>[ˈʌbˌløˀsə]</v>
       </c>
       <c r="I5" t="str">
-        <v/>
+        <v>https://static.ordnet.dk/mp3/11037/11037569_1.mp3</v>
       </c>
       <c r="J5" t="str">
-        <v/>
+        <v>ophæve sammenhængen i en helhed eller gruppe så den ophører med at eksistere</v>
       </c>
       <c r="K5" t="str">
-        <v/>
+        <v>dissolve</v>
       </c>
       <c r="L5" t="str">
         <v/>
@@ -754,7 +757,7 @@
         <v/>
       </c>
       <c r="Q5" t="str">
-        <v>pending</v>
+        <v>ok</v>
       </c>
       <c r="R5" t="str">
         <v/>
@@ -786,28 +789,28 @@
         <v>fatter</v>
       </c>
       <c r="D6" t="str">
-        <v/>
+        <v>fatter</v>
       </c>
       <c r="E6" t="str">
-        <v/>
+        <v>substantiv</v>
       </c>
       <c r="F6" t="str">
-        <v/>
+        <v>en</v>
       </c>
       <c r="G6" t="str">
-        <v/>
+        <v>-en</v>
       </c>
       <c r="H6" t="str">
-        <v/>
+        <v>[ˈfadʌ]</v>
       </c>
       <c r="I6" t="str">
-        <v/>
+        <v>https://static.ordnet.dk/mp3/11012/11012506_1.mp3</v>
       </c>
       <c r="J6" t="str">
-        <v/>
+        <v>bruges kærligt eller spøgende ved tiltale til eller omtale af ens mand eller far</v>
       </c>
       <c r="K6" t="str">
-        <v/>
+        <v>grasp</v>
       </c>
       <c r="L6" t="str">
         <v/>
@@ -825,7 +828,7 @@
         <v/>
       </c>
       <c r="Q6" t="str">
-        <v>pending</v>
+        <v>ok</v>
       </c>
       <c r="R6" t="str">
         <v/>

</xml_diff>

<commit_message>
Add phrase "Det her det ender galt" to Sange.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Sange.xlsx
+++ b/12-06-2026-vokab/Sange.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -858,25 +858,25 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q1"/>
+  <dimension ref="A1:Q2"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="30.83203125"/>
-    <col min="4" max="4" customWidth="1" width="36.83203125"/>
-    <col min="5" max="5" customWidth="1" width="36.83203125"/>
-    <col min="6" max="6" customWidth="1" width="50.83203125"/>
-    <col min="7" max="7" customWidth="1" width="24.83203125"/>
-    <col min="8" max="8" customWidth="1" width="24.83203125"/>
-    <col min="9" max="9" customWidth="1" width="24.83203125"/>
-    <col min="10" max="10" customWidth="1" width="18.83203125"/>
-    <col min="11" max="11" customWidth="1" width="10.83203125"/>
-    <col min="12" max="12" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="13" max="13" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="14" max="14" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="15" max="15" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="16" max="16" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="17" max="17" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col min="4" max="4" width="36.83203125" customWidth="1"/>
+    <col min="5" max="5" width="36.83203125" customWidth="1"/>
+    <col min="6" max="6" width="50.83203125" customWidth="1"/>
+    <col min="7" max="7" width="24.83203125" customWidth="1"/>
+    <col min="8" max="8" width="24.83203125" customWidth="1"/>
+    <col min="9" max="9" width="24.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="10.83203125" customWidth="1"/>
+    <col min="12" max="12" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="13" max="13" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="14" max="14" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="15" max="15" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="16" max="16" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="17" max="17" width="40.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -932,9 +932,62 @@
         <v>Candidates</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>ffa53bd6-19b4-4cd0-9f3b-9ed7370ffd45</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Det her det ender galt</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Det=The · her=here · det=the · ender=ends · galt=wrong</v>
+      </c>
+      <c r="E2" t="str">
+        <v>this it ends badly</v>
+      </c>
+      <c r="F2" t="str">
+        <v>… t komme Hvad!? Det vil de ikke tro Hvem!? De bli'r et par og resultatet er Vores trio bli'r til to Ååh Der' romatik i luften Og trolddom overalt Sådan som de to hvisker ka' jeg se Det her det ender galt - alle. Overgangen er lidt anerledes så den får vi lige tilpasset i morgen. Vi glæder os! @alle</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Fællesklang Sønderborg | Facebook</v>
+      </c>
+      <c r="H2" t="str">
+        <v>https://www.facebook.com/groups/9417595711665677</v>
+      </c>
+      <c r="I2" t="str">
+        <v>https://www.facebook.com/groups/9417595711665677#:~:text=Det%20her%20det%20ender%20galt</v>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
+        <v>ok</v>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2" t="str">
+        <v/>
+      </c>
+      <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2" t="str">
+        <v/>
+      </c>
+      <c r="Q2" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "sitrer" to Sange.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Sange.xlsx
+++ b/12-06-2026-vokab/Sange.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -399,31 +399,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W6"/>
+  <dimension ref="A1:W7"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="18.83203125"/>
-    <col min="4" max="4" customWidth="1" width="14.83203125"/>
-    <col min="5" max="5" customWidth="1" width="11.83203125"/>
-    <col min="6" max="6" customWidth="1" width="8.83203125"/>
-    <col min="7" max="7" customWidth="1" width="26.83203125"/>
-    <col min="8" max="8" customWidth="1" width="16.83203125"/>
-    <col min="9" max="9" customWidth="1" width="18.83203125"/>
-    <col min="10" max="10" customWidth="1" width="36.83203125"/>
-    <col min="11" max="11" customWidth="1" width="36.83203125"/>
-    <col min="12" max="12" customWidth="1" width="50.83203125"/>
-    <col min="13" max="13" customWidth="1" width="24.83203125"/>
-    <col min="14" max="14" customWidth="1" width="24.83203125"/>
-    <col min="15" max="15" customWidth="1" width="24.83203125"/>
-    <col min="16" max="16" customWidth="1" width="18.83203125"/>
-    <col min="17" max="17" customWidth="1" width="10.83203125"/>
-    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="23" max="23" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="26.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="36.83203125" customWidth="1"/>
+    <col min="11" max="11" width="36.83203125" customWidth="1"/>
+    <col min="12" max="12" width="50.83203125" customWidth="1"/>
+    <col min="13" max="13" width="24.83203125" customWidth="1"/>
+    <col min="14" max="14" width="24.83203125" customWidth="1"/>
+    <col min="15" max="15" width="24.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="10.83203125" customWidth="1"/>
+    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="23" max="23" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -849,9 +849,80 @@
         <v/>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>ee46ace1-7904-4624-bc26-a40d123743ad</v>
+      </c>
+      <c r="B7" t="str">
+        <v>2026-06-16</v>
+      </c>
+      <c r="C7" t="str">
+        <v>sitrer</v>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+      <c r="E7" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7" t="str">
+        <v>-r, -de, -tBøjningsformersitrersitredesitret</v>
+      </c>
+      <c r="H7" t="str">
+        <v>[ˈsidʁʌ]</v>
+      </c>
+      <c r="I7" t="str">
+        <v>https://static.ordnet.dk/mp3/11046/11046109_1.mp3</v>
+      </c>
+      <c r="J7" t="str">
+        <v>1. foretage små, hurtige, rykvise bevægelser, især som udtryk for sindsbevægelse, anstrengelse eller stærk kulde om levende væsen eller legemsdelSynonymer bævedirreOrd i nærhedenklapre af kuldeklapre tænderklapre med tændernehakke tændergyseskælve He</v>
+      </c>
+      <c r="K7" t="str">
+        <v>quivering</v>
+      </c>
+      <c r="L7" t="str">
+        <v>Fuck det Nu vælter solen ind Og fortryller alle støvkorn på min bordplade Det' helt okay at være til Luften sitrer, når jeg rører ved din overflade</v>
+      </c>
+      <c r="M7" t="str">
+        <v>det kun vigtigt hvad det er lyrics - Google Search</v>
+      </c>
+      <c r="N7" t="str">
+        <v>https://www.google.com/search?q=det+kun+vigtigt+hvad+det+er+lyrics&amp;rlz=1C1GCEU_enDK1211DK1212&amp;oq=det+&amp;gs_lcrp=EgZjaHJvbWUqDggAEEUYJxg7GIAEGIoFMg4IABBFGCcYOxiABBiKBTIGCAEQRRg5MgcIAhAAGIAEMgcIAxAAGIAEMgcIBBAAGIAEMgcIBRAAGIAEMgYIBhBFGDwyBggHEEUYPNIBCDE3ODFqMGo3qAIAsAIA&amp;sourceid=chrome&amp;ie=UTF-8</v>
+      </c>
+      <c r="O7" t="str">
+        <v>https://www.google.com/search?q=det+kun+vigtigt+hvad+det+er+lyrics&amp;rlz=1C1GCEU_enDK1211DK1212&amp;oq=det+&amp;gs_lcrp=EgZjaHJvbWUqDggAEEUYJxg7GIAEGIoFMg4IABBFGCcYOxiABBiKBTIGCAEQRRg5MgcIAhAAGIAEMgcIAxAAGIAEMgcIBBAAGIAEMgcIBRAAGIAEMgYIBhBFGDwyBggHEEUYPNIBCDE3ODFqMGo3qAIAsAIA&amp;sourceid=chrome&amp;ie=UTF-8#:~:text=sitrer</v>
+      </c>
+      <c r="P7" t="str">
+        <v/>
+      </c>
+      <c r="Q7" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R7" t="str">
+        <v/>
+      </c>
+      <c r="S7" t="str">
+        <v/>
+      </c>
+      <c r="T7" t="str">
+        <v/>
+      </c>
+      <c r="U7" t="str">
+        <v/>
+      </c>
+      <c r="V7" t="str">
+        <v/>
+      </c>
+      <c r="W7" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W7"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -860,23 +931,23 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Q2"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="36.83203125" customWidth="1"/>
-    <col min="5" max="5" width="36.83203125" customWidth="1"/>
-    <col min="6" max="6" width="50.83203125" customWidth="1"/>
-    <col min="7" max="7" width="24.83203125" customWidth="1"/>
-    <col min="8" max="8" width="24.83203125" customWidth="1"/>
-    <col min="9" max="9" width="24.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" customWidth="1"/>
-    <col min="12" max="12" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="13" max="13" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="14" max="14" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="15" max="15" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="16" max="16" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="17" max="17" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="30.83203125"/>
+    <col min="4" max="4" customWidth="1" width="36.83203125"/>
+    <col min="5" max="5" customWidth="1" width="36.83203125"/>
+    <col min="6" max="6" customWidth="1" width="50.83203125"/>
+    <col min="7" max="7" customWidth="1" width="24.83203125"/>
+    <col min="8" max="8" customWidth="1" width="24.83203125"/>
+    <col min="9" max="9" customWidth="1" width="24.83203125"/>
+    <col min="10" max="10" customWidth="1" width="18.83203125"/>
+    <col min="11" max="11" customWidth="1" width="10.83203125"/>
+    <col min="12" max="12" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="13" max="13" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="14" max="14" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="15" max="15" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="16" max="16" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="17" max="17" customWidth="1" width="40.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Add word "rører" to Sange.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Sange.xlsx
+++ b/12-06-2026-vokab/Sange.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W7"/>
+  <dimension ref="A1:W8"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -920,9 +920,80 @@
         <v/>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>737a8e71-f184-4fe6-9f2c-25a77d73f53b</v>
+      </c>
+      <c r="B8" t="str">
+        <v>2026-06-16</v>
+      </c>
+      <c r="C8" t="str">
+        <v>rører</v>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+      <c r="E8" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8" t="str">
+        <v>-r, rørte, rørtBøjningsformerrørerrørterørt</v>
+      </c>
+      <c r="H8" t="str">
+        <v>[ˈʁɶːʌ]</v>
+      </c>
+      <c r="I8" t="str">
+        <v>https://static.ordnet.dk/mp3/11044/11044214_1.mp3</v>
+      </c>
+      <c r="J8" t="str">
+        <v>1. lægge hånden på eller ved noget så der opstår fysisk kontaktSynonym berøreOrd i nærhedenkunne nåberørestrejfesnitte2tangere Henter ... Henter ... grammatikNOGEN rører (ved) NOGEN/NOGETHun nød hans kærtegn. Det var så længe siden, han sidst havde r</v>
+      </c>
+      <c r="K8" t="str">
+        <v>touches</v>
+      </c>
+      <c r="L8" t="str">
+        <v>Fuck det Nu vælter solen ind Og fortryller alle støvkorn på min bordplade Det' helt okay at være til Luften sitrer, når jeg rører ved din overflade</v>
+      </c>
+      <c r="M8" t="str">
+        <v>det kun vigtigt hvad det er lyrics - Google Search</v>
+      </c>
+      <c r="N8" t="str">
+        <v>https://www.google.com/search?q=det+kun+vigtigt+hvad+det+er+lyrics&amp;rlz=1C1GCEU_enDK1211DK1212&amp;oq=det+&amp;gs_lcrp=EgZjaHJvbWUqDggAEEUYJxg7GIAEGIoFMg4IABBFGCcYOxiABBiKBTIGCAEQRRg5MgcIAhAAGIAEMgcIAxAAGIAEMgcIBBAAGIAEMgcIBRAAGIAEMgYIBhBFGDwyBggHEEUYPNIBCDE3ODFqMGo3qAIAsAIA&amp;sourceid=chrome&amp;ie=UTF-8</v>
+      </c>
+      <c r="O8" t="str">
+        <v>https://www.google.com/search?q=det+kun+vigtigt+hvad+det+er+lyrics&amp;rlz=1C1GCEU_enDK1211DK1212&amp;oq=det+&amp;gs_lcrp=EgZjaHJvbWUqDggAEEUYJxg7GIAEGIoFMg4IABBFGCcYOxiABBiKBTIGCAEQRRg5MgcIAhAAGIAEMgcIAxAAGIAEMgcIBBAAGIAEMgcIBRAAGIAEMgYIBhBFGDwyBggHEEUYPNIBCDE3ODFqMGo3qAIAsAIA&amp;sourceid=chrome&amp;ie=UTF-8#:~:text=r%C3%B8rer</v>
+      </c>
+      <c r="P8" t="str">
+        <v/>
+      </c>
+      <c r="Q8" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R8" t="str">
+        <v/>
+      </c>
+      <c r="S8" t="str">
+        <v/>
+      </c>
+      <c r="T8" t="str">
+        <v/>
+      </c>
+      <c r="U8" t="str">
+        <v/>
+      </c>
+      <c r="V8" t="str">
+        <v/>
+      </c>
+      <c r="W8" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W8"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>